<commit_message>
Align May budget summary with exclude VAT
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2026/PP-2605 Monthly Budget Application Form.xlsx
+++ b/2026/PP-2605 Monthly Budget Application Form.xlsx
@@ -5397,7 +5397,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5486,8 +5486,8 @@
         <v>0</v>
       </c>
       <c r="E4" s="130">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>53782</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>44818</v>
       </c>
       <c r="F4" s="130">
         <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
@@ -5499,7 +5499,7 @@
       </c>
       <c r="H4" s="140">
         <f t="shared" ref="H4:H10" si="1">SUM(E4:F4)</f>
-        <v>70195</v>
+        <v>61231</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
@@ -5516,7 +5516,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="130">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F5" s="130">
@@ -5546,7 +5546,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="130">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F6" s="130">
@@ -5576,7 +5576,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="130">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F7" s="130">
@@ -5606,7 +5606,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="130">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F8" s="130">
@@ -5636,8 +5636,8 @@
         <v>0</v>
       </c>
       <c r="E9" s="130">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>32400</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>27000</v>
       </c>
       <c r="F9" s="130">
         <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
@@ -5649,7 +5649,7 @@
       </c>
       <c r="H9" s="140">
         <f t="shared" si="1"/>
-        <v>32400</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
@@ -5666,7 +5666,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="130">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F10" s="130">
@@ -5696,8 +5696,8 @@
         <v>0</v>
       </c>
       <c r="E11" s="138">
-        <f t="shared" si="2"/>
-        <v>86182</v>
+        <f t="shared" si="2">SUM(E4:E10)</f>
+        <v>71818</v>
       </c>
       <c r="F11" s="138">
         <f t="shared" si="2"/>
@@ -5708,8 +5708,8 @@
         <v>0</v>
       </c>
       <c r="H11" s="141">
-        <f t="shared" si="2"/>
-        <v>104895</v>
+        <f t="shared" si="2">SUM(H4:H10)</f>
+        <v>90531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>